<commit_message>
Enrichir la collecte, tracer les chiffres et guider les demarches
</commit_message>
<xml_diff>
--- a/docs/dossiers/dossier-a-propos-60-m2-paris-18eme-arrondissement-63e78a32.xlsx
+++ b/docs/dossiers/dossier-a-propos-60-m2-paris-18eme-arrondissement-63e78a32.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Annonce" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Synthèse'!$A$1:$C$61</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Synthèse'!$A$1:$C$58</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -27,7 +27,7 @@
     <numFmt numFmtId="167" formatCode="0.0"/>
     <numFmt numFmtId="168" formatCode="#,##0&quot; €/mois&quot;"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -71,11 +71,6 @@
       <name val="Calibri"/>
       <b val="1"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="0098351B"/>
-      <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -140,7 +135,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
@@ -154,11 +149,11 @@
       <alignment vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="10" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="10" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -176,17 +171,14 @@
     <xf numFmtId="168" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -801,7 +793,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F60"/>
+  <dimension ref="A1:F57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -841,7 +833,7 @@
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>Dossier généré le 25/10/2026 — indicatif, l'offre de prêt de la banque fait foi.</t>
+          <t>Dossier généré le 26/10/2026 — indicatif, l'offre de prêt de la banque fait foi.</t>
         </is>
       </c>
     </row>
@@ -937,7 +929,7 @@
     <row r="13">
       <c r="A13" s="13" t="inlineStr">
         <is>
-          <t>EN CLAIR — Sur la base d'un loyer ESTIMÉ (pas de bail signé à ce stade) : aux hypothèses de ce dossier (apport 20 %, crédit 5,34 % sur 20 ans, charges provisionnées), le bien s'autofinance : le loyer couvre crédit et charges et laisse environ +383 €/mois.</t>
+          <t>EN CLAIR — Sur la base d'un loyer ESTIMÉ (pas de bail signé à ce stade) : aux hypothèses de ce dossier (apport 20 %, crédit 5,34 % sur 20 ans, charges provisionnées), le bien s'autofinance : le loyer couvre crédit et charges et laisse environ +178 €/mois.</t>
         </is>
       </c>
     </row>
@@ -999,7 +991,7 @@
         </is>
       </c>
       <c r="B20" s="18" t="n">
-        <v>1736</v>
+        <v>1500</v>
       </c>
       <c r="C20" s="19" t="inlineStr">
         <is>
@@ -1395,7 +1387,7 @@
       </c>
       <c r="B57" s="15" t="inlineStr">
         <is>
-          <t>64/100</t>
+          <t>72/100</t>
         </is>
       </c>
       <c r="C57" s="19" t="inlineStr">
@@ -1404,20 +1396,11 @@
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="27" t="inlineStr">
-        <is>
-          <t>⚠ AVERTISSEMENT : le rendement affiché par le vendeur est anormalement élevé. Exiger le bail et les quittances avant toute offre — ce dossier reprend le loyer annoncé tel quel.</t>
-        </is>
-      </c>
-    </row>
-    <row r="60"/>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="11">
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="A41:C41"/>
     <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A59:C60"/>
     <mergeCell ref="A3:C3"/>
     <mergeCell ref="A13:C14"/>
     <mergeCell ref="A34:C34"/>
@@ -1494,27 +1477,27 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="28" t="inlineStr">
+      <c r="A1" s="27" t="inlineStr">
         <is>
           <t>Année</t>
         </is>
       </c>
-      <c r="B1" s="28" t="inlineStr">
+      <c r="B1" s="27" t="inlineStr">
         <is>
           <t>Capital dû en début d'année</t>
         </is>
       </c>
-      <c r="C1" s="28" t="inlineStr">
+      <c r="C1" s="27" t="inlineStr">
         <is>
           <t>Intérêts de l'année</t>
         </is>
       </c>
-      <c r="D1" s="28" t="inlineStr">
+      <c r="D1" s="27" t="inlineStr">
         <is>
           <t>Capital remboursé</t>
         </is>
       </c>
-      <c r="E1" s="28" t="inlineStr">
+      <c r="E1" s="27" t="inlineStr">
         <is>
           <t>Capital restant dû</t>
         </is>
@@ -2187,144 +2170,144 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="29" t="inlineStr">
+      <c r="A1" s="28" t="inlineStr">
         <is>
           <t>Titre</t>
         </is>
       </c>
-      <c r="B1" s="30" t="inlineStr">
+      <c r="B1" s="29" t="inlineStr">
         <is>
           <t>cession À propos 60 m²</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="29" t="inlineStr">
+      <c r="A2" s="28" t="inlineStr">
         <is>
           <t>Lien</t>
         </is>
       </c>
-      <c r="B2" s="31" t="inlineStr">
+      <c r="B2" s="30" t="inlineStr">
         <is>
           <t>https://www.logic-immo.com/detail-vente-261896727</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="29" t="inlineStr">
+      <c r="A3" s="28" t="inlineStr">
         <is>
           <t>Ville</t>
         </is>
       </c>
-      <c r="B3" s="30" t="inlineStr">
+      <c r="B3" s="29" t="inlineStr">
         <is>
           <t>À propos 60 m² Paris 18ème arrondissement (75018)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="29" t="inlineStr">
+      <c r="A4" s="28" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="B4" s="30" t="inlineStr">
+      <c r="B4" s="29" t="inlineStr">
         <is>
           <t>alerte_logic_immo</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="29" t="inlineStr">
+      <c r="A5" s="28" t="inlineStr">
         <is>
           <t>Première détection</t>
         </is>
       </c>
-      <c r="B5" s="30" t="inlineStr">
+      <c r="B5" s="29" t="inlineStr">
         <is>
           <t>2026-09-07</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="29" t="inlineStr">
+      <c r="A6" s="28" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="B6" s="30" t="inlineStr">
+      <c r="B6" s="29" t="inlineStr">
         <is>
           <t>Murs libres</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="29" t="inlineStr">
+      <c r="A7" s="28" t="inlineStr">
         <is>
           <t>Caractéristiques</t>
         </is>
       </c>
-      <c r="B7" s="30" t="inlineStr">
+      <c r="B7" s="29" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="29" t="inlineStr">
+      <c r="A8" s="28" t="inlineStr">
         <is>
           <t>Évolution du prix</t>
         </is>
       </c>
-      <c r="B8" s="30" t="inlineStr">
+      <c r="B8" s="29" t="inlineStr">
         <is>
           <t>stable depuis la première vue</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="29" t="inlineStr">
+      <c r="A9" s="28" t="inlineStr">
         <is>
           <t>Fourchette de marché</t>
         </is>
       </c>
-      <c r="B9" s="30" t="inlineStr">
+      <c r="B9" s="29" t="inlineStr">
         <is>
           <t>468 ventes réelles 2023-2025 (DVF)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="29" t="inlineStr">
+      <c r="A10" s="28" t="inlineStr">
         <is>
           <t>Lecture du prix</t>
         </is>
       </c>
-      <c r="B10" s="30" t="inlineStr">
+      <c r="B10" s="29" t="inlineStr">
         <is>
           <t>Décote sans explication visible dans l'annonce : possible bonne affaire — ou défaut caché (état, copropriété, bail) à vérifier sur place.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="29" t="inlineStr">
+      <c r="A11" s="28" t="inlineStr">
         <is>
           <t>Alertes</t>
         </is>
       </c>
-      <c r="B11" s="30" t="inlineStr">
-        <is>
-          <t>localisation_incoherente · loyer_estime · rendement_anormalement_eleve</t>
+      <c r="B11" s="29" t="inlineStr">
+        <is>
+          <t>localisation_incoherente · loyer_estime · occupation_a_confirmer</t>
         </is>
       </c>
     </row>
     <row r="12" ht="110" customHeight="1">
-      <c r="A12" s="29" t="inlineStr">
+      <c r="A12" s="28" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="B12" s="30" t="inlineStr">
+      <c r="B12" s="29" t="inlineStr">
         <is>
           <t>190 000 € Hôtel / Restaurant 60 m² Paris 18ème arrondissement (75018) Groupe POINTdeVENTE Voir l'annonce</t>
         </is>

</xml_diff>